<commit_message>
varias modificaciones x el usuario
</commit_message>
<xml_diff>
--- a/public/informes-templates/INFORME ADICIONAL  .xlsx
+++ b/public/informes-templates/INFORME ADICIONAL  .xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{514FD4D7-833F-4AA4-80C5-64B7042E906B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA689243-ED69-46E0-B646-D0390B20FBC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,7 +87,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +145,12 @@
       <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -329,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -345,81 +351,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -447,6 +378,78 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -673,16 +676,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="14"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="20"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
@@ -703,14 +706,14 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="26"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="28"/>
+      <c r="A2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="33"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
@@ -731,14 +734,14 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="25"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="30"/>
+      <c r="A3" s="34"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="36"/>
       <c r="I3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -758,14 +761,14 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="20"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="21"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -786,18 +789,18 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="11"/>
-      <c r="E5" s="22" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="16"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="11"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="16"/>
+      <c r="H5" s="17"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -889,14 +892,14 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="23"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="11"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16"/>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="16"/>
+      <c r="H8" s="17"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -917,14 +920,14 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="31"/>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="32" t="s">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="7" t="s">
         <v>21</v>
       </c>
       <c r="I9" s="1"/>
@@ -947,14 +950,14 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="36"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="36"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="11"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -975,14 +978,14 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
-      <c r="B11" s="35"/>
-      <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="36"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="11"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
@@ -1003,14 +1006,14 @@
       <c r="Z11" s="1"/>
     </row>
     <row r="12" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="36"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="11"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
@@ -1031,14 +1034,14 @@
       <c r="Z12" s="1"/>
     </row>
     <row r="13" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="34"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="36"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="10"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="11"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
@@ -1059,14 +1062,14 @@
       <c r="Z13" s="1"/>
     </row>
     <row r="14" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="35"/>
-      <c r="D14" s="36"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="36"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="11"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
@@ -1087,14 +1090,14 @@
       <c r="Z14" s="1"/>
     </row>
     <row r="15" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="34"/>
-      <c r="B15" s="35"/>
-      <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="34"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="36"/>
+      <c r="A15" s="9"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="11"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -1115,14 +1118,14 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
-      <c r="B16" s="35"/>
-      <c r="C16" s="35"/>
-      <c r="D16" s="36"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="36"/>
+      <c r="A16" s="9"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="11"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -1143,14 +1146,14 @@
       <c r="Z16" s="1"/>
     </row>
     <row r="17" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="34"/>
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="34"/>
-      <c r="F17" s="35"/>
-      <c r="G17" s="35"/>
-      <c r="H17" s="36"/>
+      <c r="A17" s="9"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="11"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -1171,14 +1174,14 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="36"/>
-      <c r="E18" s="34"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="36"/>
+      <c r="A18" s="9"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="11"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -1199,14 +1202,14 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="34"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="36"/>
+      <c r="A19" s="9"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="11"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
@@ -1227,14 +1230,14 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="37"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="37"/>
-      <c r="F20" s="38"/>
-      <c r="G20" s="38"/>
-      <c r="H20" s="39"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="14"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
@@ -1255,18 +1258,18 @@
       <c r="Z20" s="1"/>
     </row>
     <row r="21" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="11"/>
-      <c r="E21" s="17" t="s">
+      <c r="B21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="11"/>
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="17"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
@@ -1287,16 +1290,16 @@
       <c r="Z21" s="1"/>
     </row>
     <row r="22" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="11"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="17"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
@@ -1320,14 +1323,14 @@
       <c r="A23" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="11"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
+      <c r="F23" s="16"/>
+      <c r="G23" s="17"/>
       <c r="H23" s="4" t="s">
         <v>11</v>
       </c>
@@ -1354,14 +1357,14 @@
       <c r="A24" s="5">
         <v>1</v>
       </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="11"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="16"/>
+      <c r="F24" s="16"/>
+      <c r="G24" s="17"/>
       <c r="H24" s="5"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -1386,14 +1389,14 @@
       <c r="A25" s="5">
         <v>2</v>
       </c>
-      <c r="B25" s="9" t="s">
+      <c r="B25" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="11"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="17"/>
       <c r="H25" s="5"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
@@ -1418,14 +1421,14 @@
       <c r="A26" s="5">
         <v>3</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="B26" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="11"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="17"/>
       <c r="H26" s="5"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
@@ -1450,14 +1453,14 @@
       <c r="A27" s="5">
         <v>4</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="B27" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="11"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="17"/>
       <c r="H27" s="5"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
@@ -1482,14 +1485,14 @@
       <c r="A28" s="5">
         <v>5</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="B28" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="11"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="16"/>
+      <c r="E28" s="16"/>
+      <c r="F28" s="16"/>
+      <c r="G28" s="17"/>
       <c r="H28" s="5"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
@@ -1514,14 +1517,14 @@
       <c r="A29" s="5">
         <v>6</v>
       </c>
-      <c r="B29" s="9" t="s">
+      <c r="B29" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="11"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+      <c r="G29" s="17"/>
       <c r="H29" s="5"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
@@ -1546,14 +1549,14 @@
       <c r="A30" s="5">
         <v>7</v>
       </c>
-      <c r="B30" s="9" t="s">
+      <c r="B30" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="11"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+      <c r="G30" s="17"/>
       <c r="H30" s="5"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
@@ -1575,16 +1578,16 @@
       <c r="Z30" s="1"/>
     </row>
     <row r="31" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="29" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13"/>
-      <c r="F31" s="13"/>
-      <c r="G31" s="13"/>
-      <c r="H31" s="14"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="19"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19"/>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19"/>
+      <c r="H31" s="20"/>
       <c r="I31" s="1"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
@@ -1605,14 +1608,14 @@
       <c r="Z31" s="1"/>
     </row>
     <row r="32" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="15"/>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
-      <c r="D32" s="13"/>
-      <c r="E32" s="13"/>
-      <c r="F32" s="13"/>
-      <c r="G32" s="13"/>
-      <c r="H32" s="14"/>
+      <c r="A32" s="30"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="19"/>
+      <c r="F32" s="19"/>
+      <c r="G32" s="19"/>
+      <c r="H32" s="20"/>
       <c r="I32" s="1"/>
       <c r="J32" s="1"/>
       <c r="K32" s="1"/>
@@ -1633,14 +1636,14 @@
       <c r="Z32" s="1"/>
     </row>
     <row r="33" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="11"/>
+      <c r="A33" s="15"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16"/>
+      <c r="D33" s="16"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="17"/>
       <c r="I33" s="1"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
@@ -1661,14 +1664,14 @@
       <c r="Z33" s="1"/>
     </row>
     <row r="34" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="6"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
-      <c r="H34" s="8"/>
+      <c r="A34" s="37"/>
+      <c r="B34" s="37"/>
+      <c r="C34" s="37"/>
+      <c r="D34" s="37"/>
+      <c r="E34" s="37"/>
+      <c r="F34" s="37"/>
+      <c r="G34" s="37"/>
+      <c r="H34" s="38"/>
       <c r="I34" s="1"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
@@ -1689,14 +1692,14 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="16"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="11"/>
+      <c r="A35" s="15"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="17"/>
       <c r="I35" s="1"/>
       <c r="J35" s="1"/>
       <c r="K35" s="1"/>
@@ -1717,14 +1720,14 @@
       <c r="Z35" s="1"/>
     </row>
     <row r="36" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="16"/>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10"/>
-      <c r="H36" s="11"/>
+      <c r="A36" s="15"/>
+      <c r="B36" s="16"/>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+      <c r="H36" s="17"/>
       <c r="I36" s="1"/>
       <c r="J36" s="1"/>
       <c r="K36" s="1"/>
@@ -5609,18 +5612,12 @@
       <c r="Z174" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
-    <mergeCell ref="A2:H3"/>
+  <mergeCells count="23">
     <mergeCell ref="A36:H36"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="E5:H5"/>
     <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="E21:H21"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="B23:G23"/>
     <mergeCell ref="B24:G24"/>
     <mergeCell ref="B25:G25"/>
     <mergeCell ref="B26:G26"/>
@@ -5632,6 +5629,13 @@
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="A33:H33"/>
     <mergeCell ref="A35:H35"/>
+    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="E21:H21"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="A2:H3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>